<commit_message>
fix: resolve React hook order violation in Phase5 and fix jspdf import in Phase6
</commit_message>
<xml_diff>
--- a/app_unified/public/PUMPS (1).xlsx
+++ b/app_unified/public/PUMPS (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Desktop\ESP DESING ESTUDIO\app_unified\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B14C00D-FB13-4B80-8E5B-B47FC74BDB33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B77EDF17-8B40-4407-B648-A76108D461D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{FC341EB1-65C7-47F8-9E2D-590F22EBE9EA}"/>
   </bookViews>
@@ -18,8 +18,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">MOTORS!$A$3:$AH$293</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">PUMP!$A$2:$AJ$2</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -312,7 +313,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1553" uniqueCount="640">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1555" uniqueCount="641">
   <si>
     <t>Required Pump data</t>
   </si>
@@ -2285,6 +2286,9 @@
   <si>
     <t>4.31E-20</t>
   </si>
+  <si>
+    <t>WE2700</t>
+  </si>
 </sst>
 </file>
 
@@ -19293,72 +19297,102 @@
       <c r="AF161" s="98"/>
     </row>
     <row r="162" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A162" s="32"/>
-      <c r="B162" s="27"/>
-      <c r="C162" s="33"/>
-      <c r="D162" s="27"/>
-      <c r="E162" s="27"/>
-      <c r="F162" s="27"/>
-      <c r="G162" s="27"/>
-      <c r="H162" s="27"/>
-      <c r="I162" s="24"/>
-      <c r="J162" s="27"/>
-      <c r="K162" s="24"/>
-      <c r="L162" s="24"/>
-      <c r="M162" s="24"/>
-      <c r="N162" s="24"/>
-      <c r="O162" s="24"/>
-      <c r="P162" s="24"/>
-      <c r="Q162" s="24"/>
-      <c r="R162" s="24"/>
-      <c r="S162" s="24"/>
-      <c r="T162" s="24"/>
-      <c r="U162" s="24"/>
-      <c r="V162" s="24"/>
-      <c r="W162" s="29"/>
-      <c r="X162" s="30"/>
-      <c r="Y162" s="30"/>
-      <c r="Z162" s="26"/>
-      <c r="AA162" s="30"/>
-      <c r="AB162" s="30"/>
-      <c r="AC162" s="31"/>
-      <c r="AD162" s="31"/>
-      <c r="AE162" s="31"/>
-      <c r="AF162" s="36"/>
-    </row>
-    <row r="163" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A163" s="32"/>
-      <c r="B163" s="27"/>
-      <c r="C163" s="33"/>
-      <c r="D163" s="27"/>
-      <c r="E163" s="27"/>
-      <c r="F163" s="27"/>
-      <c r="G163" s="27"/>
-      <c r="H163" s="27"/>
-      <c r="I163" s="27"/>
-      <c r="J163" s="27"/>
-      <c r="K163" s="24"/>
-      <c r="L163" s="24"/>
-      <c r="M163" s="24"/>
-      <c r="N163" s="24"/>
-      <c r="O163" s="24"/>
-      <c r="P163" s="125"/>
-      <c r="Q163" s="24"/>
-      <c r="R163" s="24"/>
-      <c r="S163" s="24"/>
-      <c r="T163" s="24"/>
-      <c r="U163" s="125"/>
-      <c r="V163" s="24"/>
-      <c r="W163" s="29"/>
-      <c r="X163" s="30"/>
-      <c r="Y163" s="30"/>
-      <c r="Z163" s="26"/>
-      <c r="AA163" s="30"/>
-      <c r="AB163" s="30"/>
-      <c r="AC163" s="31"/>
-      <c r="AD163" s="31"/>
-      <c r="AE163" s="31"/>
-      <c r="AF163" s="36"/>
+      <c r="A162" s="14" t="s">
+        <v>523</v>
+      </c>
+      <c r="B162" s="93">
+        <v>538</v>
+      </c>
+      <c r="C162" s="93" t="s">
+        <v>640</v>
+      </c>
+      <c r="D162" s="93">
+        <v>300</v>
+      </c>
+      <c r="E162" s="93">
+        <v>2716</v>
+      </c>
+      <c r="F162" s="93">
+        <v>3500</v>
+      </c>
+      <c r="G162" s="93">
+        <v>0.7</v>
+      </c>
+      <c r="H162" s="93">
+        <v>71.709999999999994</v>
+      </c>
+      <c r="I162" s="93">
+        <v>4850</v>
+      </c>
+      <c r="J162" s="72">
+        <v>60</v>
+      </c>
+      <c r="K162" s="78">
+        <v>71.7</v>
+      </c>
+      <c r="L162" s="78">
+        <v>-6.6800000000000002E-3</v>
+      </c>
+      <c r="M162" s="78">
+        <v>6.9600000000000003E-6</v>
+      </c>
+      <c r="N162" s="78">
+        <v>-4.6800000000000004E-9</v>
+      </c>
+      <c r="O162" s="78">
+        <v>9.8800000000000003E-13</v>
+      </c>
+      <c r="P162" s="78">
+        <v>-7.9900000000000002E-17</v>
+      </c>
+      <c r="Q162" s="44">
+        <v>0.90600000000000003</v>
+      </c>
+      <c r="R162" s="78">
+        <v>2.7500000000000001E-5</v>
+      </c>
+      <c r="S162" s="78">
+        <v>3.3799999999999998E-7</v>
+      </c>
+      <c r="T162" s="78">
+        <v>-1.7800000000000001E-10</v>
+      </c>
+      <c r="U162" s="78">
+        <v>3.7499999999999998E-14</v>
+      </c>
+      <c r="V162" s="78">
+        <v>-2.9799999999999999E-18</v>
+      </c>
+      <c r="W162" s="80">
+        <v>5.38</v>
+      </c>
+      <c r="X162" s="100">
+        <v>5000</v>
+      </c>
+      <c r="Y162" s="100">
+        <v>6000</v>
+      </c>
+      <c r="Z162" s="82">
+        <v>0.88</v>
+      </c>
+      <c r="AA162" s="100">
+        <v>250</v>
+      </c>
+      <c r="AB162" s="100">
+        <v>400</v>
+      </c>
+      <c r="AC162" s="101">
+        <v>5</v>
+      </c>
+      <c r="AD162" s="101">
+        <v>98</v>
+      </c>
+      <c r="AE162" s="101">
+        <v>7</v>
+      </c>
+      <c r="AF162" s="98">
+        <v>18000</v>
+      </c>
     </row>
     <row r="164" spans="1:34" s="44" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="32"/>
@@ -51512,16 +51546,17 @@
       <c r="AG1104" s="36"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:AJ2" xr:uid="{053E6D0B-9E01-4484-8758-0E93695A87D4}"/>
   <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter 1 for gas handler" sqref="AH5:AH117" xr:uid="{D4F63CA9-4B8A-4E8D-8A06-46E288212DB9}">
       <formula1>$A$1000:$A$1001</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter 1 for obsolete" sqref="AG5:AG117 AF152:AF178 AF118:AF149 AG179:AG1103" xr:uid="{6AE47EA0-4762-42E9-B62C-07E716141A03}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Enter 1 for obsolete" sqref="AG5:AG117 AF118:AF149 AG179:AG1103 AF152:AF162 AF164:AF178" xr:uid="{6AE47EA0-4762-42E9-B62C-07E716141A03}">
       <formula1>$A$1000:$A$1001</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Important Notice:" prompt="If a manufacturer is not the SubPUMP databank, this field is required. The available manufacturers within SubPUMP can be found in the drop down list in the manufacturer field (Column B)." sqref="W39 W82:W97 W7:W34 W42:W77 W79:W80 W99:W100 W103:W117" xr:uid="{3ABA8888-4F6D-4392-92AF-AB8BE0A86DDD}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Important Notice:" prompt="-------_x000a_If a manufacturer is not in SubPUMP databank, this field is required._x000a_-------_x000a_Manufacturers in SubPUMP:_x000a_Almaz, Alnas, Borets, CAI, Centrilift/ODI or CLift, ESP, Lemaz, Novomet, Novo, ODI, Schlumberger/Reda or Reda, Weatherford or Wford, WSP" sqref="W179:W1103 V175:V178 V118:V149 V161:V173 W159 V152:V158" xr:uid="{9A547A56-E420-4C2C-BE7C-866904004891}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Manufacturer Name" prompt="Select a manufacturer from the list, or enter a new manufacturer using a short name" sqref="B179:B1103 A153 A155:A160 A162:A178" xr:uid="{730E29A7-E193-4760-8A9E-D7881A70E46B}">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Important Notice:" prompt="-------_x000a_If a manufacturer is not in SubPUMP databank, this field is required._x000a_-------_x000a_Manufacturers in SubPUMP:_x000a_Almaz, Alnas, Borets, CAI, Centrilift/ODI or CLift, ESP, Lemaz, Novomet, Novo, ODI, Schlumberger/Reda or Reda, Weatherford or Wford, WSP" sqref="W179:W1103 V175:V178 V118:V149 W159 V152:V158 W162 V161:V162 V164:V173" xr:uid="{9A547A56-E420-4C2C-BE7C-866904004891}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Manufacturer Name" prompt="Select a manufacturer from the list, or enter a new manufacturer using a short name" sqref="B179:B1103 A153 A155:A160 A162 A164:A178" xr:uid="{730E29A7-E193-4760-8A9E-D7881A70E46B}">
       <formula1>$A$1009:$A$1021</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
fix: resolve jspdf and html2canvas via Vite aliases to CDN for fully automatic dependency resolution
</commit_message>
<xml_diff>
--- a/app_unified/public/PUMPS (1).xlsx
+++ b/app_unified/public/PUMPS (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\OneDrive\Desktop\ESP DESING ESTUDIO\app_unified\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B77EDF17-8B40-4407-B648-A76108D461D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13EF2173-DF3D-4E0B-9B95-B2ED56E31FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{FC341EB1-65C7-47F8-9E2D-590F22EBE9EA}"/>
   </bookViews>
@@ -2287,7 +2287,7 @@
     <t>4.31E-20</t>
   </si>
   <si>
-    <t>WE2700</t>
+    <t>WE-2700</t>
   </si>
 </sst>
 </file>

</xml_diff>